<commit_message>
Webhook → Direct SSG Script Conversions
1. All apis have been converted to script
2. added course run date sync log
(to be improved)
</commit_message>
<xml_diff>
--- a/public/ssg_templates/Course_Run_Template.xlsx
+++ b/public/ssg_templates/Course_Run_Template.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBACB681-7103-4CF7-A741-B4524A8F5249}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EDE016D-6DE5-4A04-97D8-063F54EC31C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4464" yWindow="0" windowWidth="16080" windowHeight="12360" tabRatio="599" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="599" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Course Runs Upload Template" sheetId="4" r:id="rId1"/>
     <sheet name="Definition" sheetId="5" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Course Runs Upload Template'!$A$1:$AQ$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Course Runs Upload Template'!$A$1:$AL$1</definedName>
     <definedName name="Session_End_Date">'Course Runs Upload Template'!$W$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="137">
   <si>
     <t>Attribute</t>
   </si>
@@ -172,43 +172,6 @@
   </si>
   <si>
     <t>This field is used to enter the email of the trainer</t>
-  </si>
-  <si>
-    <t>Key Domain / Sector Areas of Practice</t>
-  </si>
-  <si>
-    <t>This field used to indicate the Key Domain / Sector Areas of Practice of the trainer. 
-For existing trainer, leave this field empty.</t>
-  </si>
-  <si>
-    <t>X(1000)</t>
-  </si>
-  <si>
-    <t>Qualification Level</t>
-  </si>
-  <si>
-    <t>This field used to indicate the qualification level of the trainer. 
-For existing trainer, leave this field empty.</t>
-  </si>
-  <si>
-    <t>X(2)</t>
-  </si>
-  <si>
-    <t>Refer to SSEC-EQA Level 2 Code</t>
-  </si>
-  <si>
-    <t>Qualification Description</t>
-  </si>
-  <si>
-    <t>This field used to indicate the qualification description of the trainer. 
-For existing trainer, leave this field empty.</t>
-  </si>
-  <si>
-    <t>Experience</t>
-  </si>
-  <si>
-    <t>This field used to enter the experience of the trainer. 
-For existing trainer, leave this field empty.</t>
   </si>
   <si>
     <t xml:space="preserve">Note: </t>
@@ -712,9 +675,6 @@
     <t>Trainer ID Type</t>
   </si>
   <si>
-    <t>Trainer Role</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">This field used to indicate the type of trainer as "Existing" or "New". Select the value from dropdown.
  </t>
@@ -752,10 +712,6 @@
     <t>This is a dropdown field for selecting one of the five ID Type.
 Possible values : 
 Singapore Pink Card,Singapore Blue Card, FIN/Work Permit,Foreign Passport,Others</t>
-  </si>
-  <si>
-    <t>This is a dropdown field for selecting Role Type.
-Possible values : Trainer, Assessor and Trainer and Assessor</t>
   </si>
   <si>
     <t>7.Course run creation for WSQ Competency Standards accredited courses is no longer allowed for runs ending beyond 31 December 2022.</t>
@@ -859,6 +815,57 @@
       <t xml:space="preserve">
 This field is only applicable to Training Providers who are whitelisted to provide the Course Application URL.</t>
     </r>
+  </si>
+  <si>
+    <t>TGS-2021002504</t>
+  </si>
+  <si>
+    <t>Vibe Coding for Agentic AI Workflows and Responsive Web UI</t>
+  </si>
+  <si>
+    <t>20261026</t>
+  </si>
+  <si>
+    <t>20261027</t>
+  </si>
+  <si>
+    <t>20261028</t>
+  </si>
+  <si>
+    <t>1 Classroom Facilitated Training</t>
+  </si>
+  <si>
+    <t>2 Asynchronous E-learning</t>
+  </si>
+  <si>
+    <t>4 On the Job Training</t>
+  </si>
+  <si>
+    <t>8 Assessment</t>
+  </si>
+  <si>
+    <t>9 Synchronous E-learning</t>
+  </si>
+  <si>
+    <t>10 Work-based/Workplace Learning</t>
+  </si>
+  <si>
+    <t>20261029</t>
+  </si>
+  <si>
+    <t>enquiry@tertiaryinfotech.com</t>
+  </si>
+  <si>
+    <t>737715</t>
+  </si>
+  <si>
+    <t>07</t>
+  </si>
+  <si>
+    <t>85-87</t>
+  </si>
+  <si>
+    <t>Training room</t>
   </si>
 </sst>
 </file>
@@ -1605,7 +1612,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AQ943"/>
+  <dimension ref="A1:AR941"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="27.5546875" style="1" bestFit="1" customWidth="1"/>
@@ -1643,15 +1650,11 @@
     <col min="36" max="36" width="28.5546875" style="33" customWidth="1"/>
     <col min="37" max="37" width="20.109375" style="1" customWidth="1"/>
     <col min="38" max="38" width="20.5546875" customWidth="1"/>
-    <col min="39" max="39" width="20" style="1" customWidth="1"/>
-    <col min="40" max="40" width="25.109375" style="1" customWidth="1"/>
-    <col min="41" max="41" width="24.109375" style="1" customWidth="1"/>
-    <col min="42" max="42" width="30.88671875" style="1" customWidth="1"/>
-    <col min="43" max="43" width="28.88671875" style="1" customWidth="1"/>
-    <col min="44" max="16384" width="9.109375" style="1"/>
+    <col min="39" max="39" width="28.88671875" style="1" hidden="1" customWidth="1"/>
+    <col min="40" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" s="46" customFormat="1" ht="55.2">
+    <row r="1" spans="1:39" s="46" customFormat="1" ht="55.2">
       <c r="A1" s="34" t="s">
         <v>5</v>
       </c>
@@ -1671,28 +1674,28 @@
         <v>13</v>
       </c>
       <c r="G1" s="35" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="H1" s="35" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="I1" s="48" t="s">
-        <v>129</v>
+        <v>116</v>
       </c>
       <c r="J1" s="36" t="s">
         <v>30</v>
       </c>
       <c r="K1" s="36" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="L1" s="36" t="s">
         <v>32</v>
       </c>
       <c r="M1" s="36" t="s">
-        <v>126</v>
+        <v>113</v>
       </c>
       <c r="N1" s="36" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="O1" s="37" t="s">
         <v>18</v>
@@ -1713,22 +1716,22 @@
         <v>24</v>
       </c>
       <c r="U1" s="39" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="V1" s="40" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="W1" s="39" t="s">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="X1" s="41" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="Y1" s="41" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="Z1" s="42" t="s">
-        <v>65</v>
+        <v>54</v>
       </c>
       <c r="AA1" s="41" t="s">
         <v>27</v>
@@ -1761,102 +1764,134 @@
         <v>44</v>
       </c>
       <c r="AK1" s="45" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="AL1" s="45" t="s">
-        <v>117</v>
-      </c>
-      <c r="AM1" s="44" t="s">
-        <v>118</v>
-      </c>
-      <c r="AN1" s="44" t="s">
-        <v>46</v>
-      </c>
-      <c r="AO1" s="44" t="s">
-        <v>49</v>
-      </c>
-      <c r="AP1" s="44" t="s">
-        <v>53</v>
-      </c>
-      <c r="AQ1" s="44" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="2" spans="1:43" s="25" customFormat="1">
-      <c r="A2"/>
-      <c r="B2"/>
-      <c r="H2"/>
+        <v>106</v>
+      </c>
+      <c r="AM1" s="42"/>
+    </row>
+    <row r="2" spans="1:39" s="25" customFormat="1">
+      <c r="A2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C2" s="25" t="s">
+        <v>122</v>
+      </c>
+      <c r="D2" s="25" t="s">
+        <v>123</v>
+      </c>
+      <c r="E2" s="25" t="s">
+        <v>124</v>
+      </c>
+      <c r="F2" s="25" t="s">
+        <v>131</v>
+      </c>
+      <c r="G2" s="25" t="s">
+        <v>125</v>
+      </c>
+      <c r="H2" s="47" t="s">
+        <v>132</v>
+      </c>
       <c r="I2"/>
+      <c r="O2" s="25" t="s">
+        <v>133</v>
+      </c>
+      <c r="P2" s="25" t="s">
+        <v>134</v>
+      </c>
+      <c r="Q2" s="25" t="s">
+        <v>135</v>
+      </c>
+      <c r="R2" s="25" t="s">
+        <v>136</v>
+      </c>
+      <c r="S2" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="T2" s="25" t="s">
+        <v>6</v>
+      </c>
       <c r="AG2" s="26"/>
       <c r="AJ2" s="33"/>
       <c r="AL2"/>
-      <c r="AN2" s="26"/>
-    </row>
-    <row r="3" spans="1:43" s="25" customFormat="1">
+      <c r="AM2" s="25" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="3" spans="1:39" s="25" customFormat="1">
       <c r="A3"/>
       <c r="B3"/>
       <c r="H3"/>
       <c r="I3"/>
       <c r="AG3" s="26"/>
-      <c r="AJ3" s="33"/>
-      <c r="AL3"/>
-    </row>
-    <row r="4" spans="1:43" s="25" customFormat="1">
+      <c r="AJ3" s="47"/>
+      <c r="AL3" s="26"/>
+      <c r="AM3" s="25" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="4" spans="1:39">
       <c r="A4"/>
       <c r="B4"/>
-      <c r="H4"/>
-      <c r="I4"/>
-      <c r="AG4" s="26"/>
-      <c r="AJ4" s="47"/>
-      <c r="AL4" s="26"/>
-      <c r="AN4" s="26"/>
-      <c r="AP4" s="26"/>
-    </row>
-    <row r="5" spans="1:43">
+      <c r="AM4" s="1" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="5" spans="1:39">
       <c r="A5"/>
       <c r="B5"/>
-    </row>
-    <row r="6" spans="1:43">
+      <c r="AM5" s="1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="6" spans="1:39">
       <c r="A6"/>
       <c r="B6"/>
-    </row>
-    <row r="7" spans="1:43">
+      <c r="AM6" s="1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="7" spans="1:39">
       <c r="A7"/>
       <c r="B7"/>
     </row>
-    <row r="8" spans="1:43">
+    <row r="8" spans="1:39">
       <c r="A8"/>
       <c r="B8"/>
     </row>
-    <row r="9" spans="1:43">
+    <row r="9" spans="1:39">
       <c r="A9"/>
       <c r="B9"/>
     </row>
-    <row r="10" spans="1:43">
+    <row r="10" spans="1:39">
       <c r="A10"/>
       <c r="B10"/>
     </row>
-    <row r="11" spans="1:43">
+    <row r="11" spans="1:39">
       <c r="A11"/>
       <c r="B11"/>
     </row>
-    <row r="12" spans="1:43">
+    <row r="12" spans="1:39">
       <c r="A12"/>
       <c r="B12"/>
     </row>
-    <row r="13" spans="1:43">
+    <row r="13" spans="1:39">
       <c r="A13"/>
       <c r="B13"/>
     </row>
-    <row r="14" spans="1:43">
+    <row r="14" spans="1:39">
       <c r="A14"/>
       <c r="B14"/>
     </row>
-    <row r="15" spans="1:43">
+    <row r="15" spans="1:39">
       <c r="A15"/>
       <c r="B15"/>
     </row>
-    <row r="16" spans="1:43">
+    <row r="16" spans="1:39">
       <c r="A16"/>
       <c r="B16"/>
     </row>
@@ -2948,69 +2983,84 @@
       <c r="A288"/>
       <c r="B288"/>
     </row>
-    <row r="289" spans="1:2">
+    <row r="289" spans="1:39">
       <c r="A289"/>
       <c r="B289"/>
     </row>
-    <row r="290" spans="1:2">
+    <row r="290" spans="1:39">
       <c r="A290"/>
       <c r="B290"/>
     </row>
-    <row r="291" spans="1:2">
+    <row r="291" spans="1:39">
       <c r="A291"/>
       <c r="B291"/>
     </row>
-    <row r="292" spans="1:2">
+    <row r="292" spans="1:39">
       <c r="A292"/>
       <c r="B292"/>
     </row>
-    <row r="293" spans="1:2">
+    <row r="293" spans="1:39">
       <c r="A293"/>
       <c r="B293"/>
     </row>
-    <row r="294" spans="1:2">
+    <row r="294" spans="1:39">
       <c r="A294"/>
       <c r="B294"/>
     </row>
-    <row r="295" spans="1:2">
+    <row r="295" spans="1:39">
       <c r="A295"/>
       <c r="B295"/>
     </row>
-    <row r="296" spans="1:2">
+    <row r="296" spans="1:39">
       <c r="A296"/>
       <c r="B296"/>
     </row>
-    <row r="297" spans="1:2">
+    <row r="297" spans="1:39">
       <c r="A297"/>
       <c r="B297"/>
     </row>
-    <row r="298" spans="1:2">
+    <row r="298" spans="1:39">
       <c r="A298"/>
       <c r="B298"/>
     </row>
-    <row r="299" spans="1:2">
+    <row r="299" spans="1:39">
       <c r="A299"/>
       <c r="B299"/>
     </row>
-    <row r="300" spans="1:2">
+    <row r="300" spans="1:39">
       <c r="A300"/>
       <c r="B300"/>
-    </row>
-    <row r="301" spans="1:2">
+      <c r="AM300" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="301" spans="1:39">
       <c r="A301"/>
       <c r="B301"/>
-    </row>
-    <row r="302" spans="1:2">
+      <c r="AM301" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="302" spans="1:39">
       <c r="A302"/>
       <c r="B302"/>
-    </row>
-    <row r="303" spans="1:2">
+      <c r="AM302" s="1" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="303" spans="1:39">
       <c r="A303"/>
       <c r="B303"/>
-    </row>
-    <row r="304" spans="1:2">
+      <c r="AM303" s="1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="304" spans="1:39">
       <c r="A304"/>
       <c r="B304"/>
+      <c r="AM304" s="1" t="s">
+        <v>130</v>
+      </c>
     </row>
     <row r="305" spans="1:2">
       <c r="A305"/>
@@ -5560,24 +5610,16 @@
       <c r="A941"/>
       <c r="B941"/>
     </row>
-    <row r="942" spans="1:2">
-      <c r="A942"/>
-      <c r="B942"/>
-    </row>
-    <row r="943" spans="1:2">
-      <c r="A943"/>
-      <c r="B943"/>
-    </row>
   </sheetData>
   <dataConsolidate/>
-  <dataValidations xWindow="134" yWindow="576" count="41">
+  <dataValidations xWindow="134" yWindow="576" count="38">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please enter a 6 digit postal code." prompt="Please enter a 6 digit postal code." sqref="AA1 O1" xr:uid="{00000000-0002-0000-0100-000000000000}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please enter no more than 5 characters." prompt="Please enter no more than 5 characters." sqref="AC1" xr:uid="{00000000-0002-0000-0100-000001000000}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please select from the dropdown." prompt="Please select from the dropdown." sqref="AE1" xr:uid="{00000000-0002-0000-0100-000002000000}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please select from the dropdown." prompt="Please select from the dropdown." sqref="S1 S2:T1048576 AE2:AE1048576" xr:uid="{00000000-0002-0000-0100-000003000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please select from the dropdown." prompt="Please select from the dropdown." sqref="S1 AE2:AE1048576 S2:T1048576" xr:uid="{00000000-0002-0000-0100-000003000000}">
       <formula1>"Yes, No"</formula1>
     </dataValidation>
-    <dataValidation type="textLength" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please enter date in YYYYMMDD format." prompt="Please enter date in YYYYMMDD format." sqref="V1 V5:W1048576" xr:uid="{00000000-0002-0000-0100-000004000000}">
+    <dataValidation type="textLength" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please enter date in YYYYMMDD format." prompt="Please enter date in YYYYMMDD format." sqref="V1 V4:W1048576" xr:uid="{00000000-0002-0000-0100-000004000000}">
       <formula1>8</formula1>
       <formula2>8</formula2>
     </dataValidation>
@@ -5593,62 +5635,63 @@
       <formula1>0</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation type="textLength" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please enter date in YYYYMMDD format." prompt="Course End Date is mandatory._x000a_Please enter date in YYYYMMDD format._x000a_Registration Opening Date cannot be:_x000a_1. earlier than the current date._x000a_2. later than the Registration Closing Date._x000a_3. later than the Course Start Date." sqref="F1 F5:F63551" xr:uid="{00000000-0002-0000-0100-000008000000}">
+    <dataValidation type="textLength" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please enter date in YYYYMMDD format." prompt="Course End Date is mandatory._x000a_Please enter date in YYYYMMDD format._x000a_Registration Opening Date cannot be:_x000a_1. earlier than the current date._x000a_2. later than the Registration Closing Date._x000a_3. later than the Course Start Date." sqref="F1 F4:F63549" xr:uid="{00000000-0002-0000-0100-000008000000}">
       <formula1>8</formula1>
       <formula2>8</formula2>
     </dataValidation>
-    <dataValidation type="textLength" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please enter date in YYYYMMDD format." prompt="Course Start Date is mandatory._x000a_Please enter date in YYYYMMDD format._x000a_Registration Opening Date cannot be:_x000a_1. earlier than the current date._x000a_2. later than the Registration Closing Date._x000a_3. later than the Course Start Date." sqref="E1 E5:E63551" xr:uid="{00000000-0002-0000-0100-000009000000}">
+    <dataValidation type="textLength" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please enter date in YYYYMMDD format." prompt="Course Start Date is mandatory._x000a_Please enter date in YYYYMMDD format._x000a_Registration Opening Date cannot be:_x000a_1. earlier than the current date._x000a_2. later than the Registration Closing Date._x000a_3. later than the Course Start Date." sqref="E1 E4:E63549" xr:uid="{00000000-0002-0000-0100-000009000000}">
       <formula1>8</formula1>
       <formula2>8</formula2>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please enter no more than 66 characters." prompt="Please do not enter more than 320 characters. Email Address:_x000a_-Must have @_x000a_-EmailAddressLocalPart &lt;= 64 characters_x000a_-EmailAddressAtSign = 1 character_x000a_-EmailAddressDomain &lt;= 255 characters" sqref="AJ1:AJ1048576" xr:uid="{00000000-0002-0000-0100-00000A000000}"/>
-    <dataValidation type="textLength" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please enter date in YYYYMMDD format." prompt="Registration Closing Date is mandatory._x000a_Please enter date in YYYYMMDD format._x000a_Registration Opening Date cannot be:_x000a_1. earlier than the current date._x000a_2. later than the Registration Closing Date._x000a_3. later than the Course Start Date." sqref="D5:D63551 D1:D3 F2:F3" xr:uid="{00000000-0002-0000-0100-00000B000000}">
+    <dataValidation type="textLength" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please enter date in YYYYMMDD format." prompt="Registration Closing Date is mandatory._x000a_Please enter date in YYYYMMDD format._x000a_Registration Opening Date cannot be:_x000a_1. earlier than the current date._x000a_2. later than the Registration Closing Date._x000a_3. later than the Course Start Date." sqref="F2 D1:D2 D4:D63549" xr:uid="{00000000-0002-0000-0100-00000B000000}">
       <formula1>8</formula1>
       <formula2>8</formula2>
     </dataValidation>
-    <dataValidation type="textLength" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please enter date in YYYYMMDD format." prompt="Registration Opening Date is mandatory._x000a_Please enter date in YYYYMMDD format._x000a_Registration Opening Date cannot be:_x000a_1. earlier than the current date._x000a_2. later than the Registration Closing Date._x000a_3. later than the Course Start Date." sqref="F4 C1:C63551 E2:E4 D4 V2:W4" xr:uid="{00000000-0002-0000-0100-00000C000000}">
+    <dataValidation type="textLength" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please enter date in YYYYMMDD format." prompt="Registration Opening Date is mandatory._x000a_Please enter date in YYYYMMDD format._x000a_Registration Opening Date cannot be:_x000a_1. earlier than the current date._x000a_2. later than the Registration Closing Date._x000a_3. later than the Course Start Date." sqref="F3 D3 C1:C63549 E2:E3 V2:W3" xr:uid="{00000000-0002-0000-0100-00000C000000}">
       <formula1>8</formula1>
       <formula2>8</formula2>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Please do not enter more than 320 characters. Email Address:_x000a_-Must have @_x000a_-EmailAddressLocalPart &lt;= 64 characters_x000a_-EmailAddressAtSign = 1 character_x000a_-EmailAddressDomain &lt;= 255 characters" sqref="H1 H422:H1048576" xr:uid="{00000000-0002-0000-0100-00000D000000}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Please do not overwrite this field." sqref="A1:B1 A367:B1048576" xr:uid="{00000000-0002-0000-0100-00000E000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Please do not enter more than 320 characters. Email Address:_x000a_-Must have @_x000a_-EmailAddressLocalPart &lt;= 64 characters_x000a_-EmailAddressAtSign = 1 character_x000a_-EmailAddressDomain &lt;= 255 characters" sqref="H1 H420:H1048576" xr:uid="{00000000-0002-0000-0100-00000D000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Please do not overwrite this field." sqref="A1:B1 A365:B1048576" xr:uid="{00000000-0002-0000-0100-00000E000000}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please select from the dropdown" prompt="Please select from the dropdown" sqref="Z1" xr:uid="{00000000-0002-0000-0100-000015000000}">
+      <formula1>"Assessment,Asynchronous eLearning,Classroom,In-house,On-the-Job,Practical / Practicum,Supervised Field,Synchronous eLearning,Traineeship"</formula1>
+    </dataValidation>
+    <dataValidation type="textLength" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please enter no more than 1000 characters." prompt="Please enter no more than 1000 characters." sqref="AM1:AM300 AM302:AM1048576" xr:uid="{00000000-0002-0000-0100-000018000000}">
+      <formula1>1</formula1>
+      <formula2>1000</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please select ID Type." promptTitle="Trainer ID Type" prompt="Please select Trainer ID type. Possible values:_x000a_-Singapore Pink Identification Card_x000a_-Singapore Blue Identificaton Card_x000a_-FIN/Work Permit_x000a_-Foreign Passport_x000a_-Others" sqref="AL1" xr:uid="{00000000-0002-0000-0100-000022000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please select from the dropdown" prompt="Please select from the dropdown" sqref="G1" xr:uid="{00000000-0002-0000-0100-000024000000}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please select from the dropdown" prompt="Please select from the dropdown" sqref="G300:G1048576 G3:G299" xr:uid="{0A9DBD8E-98B5-417D-8BBE-275D4F7BAF2E}">
+      <formula1>#REF!</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please select from the dropdown" prompt="Please select from the dropdown" sqref="G2" xr:uid="{BFC8A9A5-114D-46A5-934F-7713966C76E2}">
+      <formula1>$AM$2:$AM$6</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please enter no more than 66 characters." prompt="Please do not enter more than 320 characters. Email Address:_x000a_-Must have @_x000a_-EmailAddressLocalPart &lt;= 64 characters_x000a_-EmailAddressAtSign = 1 character_x000a_-EmailAddressDomain &lt;= 255 characters" sqref="AJ1:AJ1048576" xr:uid="{00000000-0002-0000-0100-00000A000000}"/>
     <dataValidation type="textLength" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please enter no more than 66 characters." prompt="Please enter no more than 66 characters." sqref="AI1:AI1048576" xr:uid="{00000000-0002-0000-0100-00000F000000}">
       <formula1>1</formula1>
       <formula2>66</formula2>
     </dataValidation>
-    <dataValidation type="textLength" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please enter no more than 255 characters." prompt="Please enter no more than 255 characters." sqref="R1:R1048576 AD1:AD1048576" xr:uid="{00000000-0002-0000-0100-000010000000}">
+    <dataValidation type="textLength" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please enter no more than 255 characters." prompt="Please enter no more than 255 characters." sqref="AD1:AD1048576 R1:R1048576" xr:uid="{00000000-0002-0000-0100-000010000000}">
       <formula1>1</formula1>
       <formula2>255</formula2>
     </dataValidation>
-    <dataValidation type="textLength" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please enter no more than 3 characters." prompt="Please enter no more than 3 characters." sqref="P1:P1048576 AB1:AB1048576" xr:uid="{00000000-0002-0000-0100-000011000000}">
+    <dataValidation type="textLength" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please enter no more than 3 characters." prompt="Please enter no more than 3 characters." sqref="AB1:AB1048576 P1:P1048576" xr:uid="{00000000-0002-0000-0100-000011000000}">
       <formula1>1</formula1>
       <formula2>3</formula2>
     </dataValidation>
-    <dataValidation type="textLength" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please enter no more than 5 characters." prompt="Please enter no more than 5 characters." sqref="Q1:Q1048576 AC2:AC1048576" xr:uid="{00000000-0002-0000-0100-000012000000}">
+    <dataValidation type="textLength" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please enter no more than 5 characters." prompt="Please enter no more than 5 characters." sqref="AC2:AC1048576 Q1:Q1048576" xr:uid="{00000000-0002-0000-0100-000012000000}">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation type="textLength" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please enter a 6 digit postal code." prompt="Please enter a 6 digit postal code." sqref="O2:O1048576 AA2:AA1048576" xr:uid="{00000000-0002-0000-0100-000013000000}">
+    <dataValidation type="textLength" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please enter a 6 digit postal code." prompt="Please enter a 6 digit postal code." sqref="AA2:AA1048576 O2:O1048576" xr:uid="{00000000-0002-0000-0100-000013000000}">
       <formula1>6</formula1>
       <formula2>6</formula2>
     </dataValidation>
     <dataValidation type="textLength" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please enter valid time." prompt="Enter time in HH:MM format (24 Hr)," sqref="X2:X1048576" xr:uid="{00000000-0002-0000-0100-000014000000}">
       <formula1>0</formula1>
       <formula2>5</formula2>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please select from the dropdown" prompt="Please select from the dropdown" sqref="Z1" xr:uid="{00000000-0002-0000-0100-000015000000}">
-      <formula1>"Assessment,Asynchronous eLearning,Classroom,In-house,On-the-Job,Practical / Practicum,Supervised Field,Synchronous eLearning,Traineeship"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please select from the dropdown." prompt="Please select from the dropdown. Refer to the &quot;Allowed_Values&quot; worksheet to see the qualifcation description of each SSEC-EQA Level 2 code." sqref="AO1:AO1048576" xr:uid="{00000000-0002-0000-0100-000016000000}">
-      <formula1>"11,12,13,21,22,23,24,31,32,33,34,35,39,41,42,43,44,45,46,47,48,49,51,52,61,62,63,64,65,69,71,72,81,82,83,91,92,N1,N2,N3,N4,N9"</formula1>
-    </dataValidation>
-    <dataValidation type="textLength" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please enter no less than 50 characters and no more than 1000 characters." prompt="Please enter no less than 50 characters and no more than 1000 characters." sqref="AN1:AN1048576 AP4" xr:uid="{00000000-0002-0000-0100-000017000000}">
-      <formula1>50</formula1>
-      <formula2>1000</formula2>
-    </dataValidation>
-    <dataValidation type="textLength" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please enter no more than 1000 characters." prompt="Please enter no more than 1000 characters." sqref="AQ1:AQ1048576 AP1:AP3 AP5:AP1048576" xr:uid="{00000000-0002-0000-0100-000018000000}">
-      <formula1>1</formula1>
-      <formula2>1000</formula2>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please select from the dropdown." prompt="Please select from the dropdown." sqref="AG1:AG1048576" xr:uid="{00000000-0002-0000-0100-000019000000}">
       <formula1>"No, Yes"</formula1>
@@ -5663,36 +5706,30 @@
       <formula1>"Mr, Ms, Mdm, Mrs, Dr, Prof, Others, Miss"</formula1>
     </dataValidation>
     <dataValidation allowBlank="1" showInputMessage="1" sqref="J1:K1048576" xr:uid="{00000000-0002-0000-0100-00001D000000}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please enter no more than 66 characters." prompt="Please select Trainer Role. Possible values:_x000a_-Trainer_x000a_-Assessor_x000a_-Trainer and Assessor" sqref="AM2:AM1048576" xr:uid="{00000000-0002-0000-0100-00001E000000}">
-      <formula1>"Trainer, Assessor, Trainer and Assessor"</formula1>
-    </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please enter no more than 66 characters." prompt="Please select Trainer Role. Possible values:_x000a_-Trainer_x000a_-Assessor_x000a_-Trainer and Assessor" sqref="AM1" xr:uid="{00000000-0002-0000-0100-00001F000000}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Trainer ID Number" prompt="NRIC or FIN number or any other identification number." sqref="AK1:AK1048576" xr:uid="{00000000-0002-0000-0100-000020000000}"/>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please select ID Type." promptTitle="Trainer ID Type" prompt="Please select Trainer ID type. Possible values:_x000a_-Singapore Pink Identification Card_x000a_-Singapore Blue Identificaton Card_x000a_-FIN/Work Permit_x000a_-Foreign Passport_x000a_-Others" sqref="AL2:AL1048576" xr:uid="{00000000-0002-0000-0100-000021000000}">
       <formula1>"Singapore Pink Identification Card,Singapore Blue Identification Card,FIN/Work Permit,Foreign Passport,Others"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please select ID Type." promptTitle="Trainer ID Type" prompt="Please select Trainer ID type. Possible values:_x000a_-Singapore Pink Identification Card_x000a_-Singapore Blue Identificaton Card_x000a_-FIN/Work Permit_x000a_-Foreign Passport_x000a_-Others" sqref="AL1" xr:uid="{00000000-0002-0000-0100-000022000000}"/>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" prompt="This field is only applicable to Training Providers who are whitelisted to provide the Course Application URL." sqref="N1:N1048576" xr:uid="{00000000-0002-0000-0100-000023000000}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please select from the dropdown" prompt="Please select from the dropdown" sqref="G1" xr:uid="{00000000-0002-0000-0100-000024000000}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter up to 20 recipient email addresses, separated by semicolons ( ; ). Example: john.doe@example.com;jane.smith@example.com" sqref="I1:I1048576 H2:H421" xr:uid="{00000000-0002-0000-0100-000025000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter up to 20 recipient email addresses, separated by semicolons ( ; ). Example: john.doe@example.com;jane.smith@example.com" sqref="H2:H419 I1:I1048576" xr:uid="{00000000-0002-0000-0100-000025000000}"/>
     <dataValidation allowBlank="1" showInputMessage="1" prompt="This field is only applicable to Training Providers who are whitelisted to provide the Course Application URL." sqref="M1:M1048576" xr:uid="{00000000-0002-0000-0100-000026000000}"/>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Z2:Z1048576" xr:uid="{799B964E-9462-499B-991E-97C997B6ED91}">
       <formula1>#REF!</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please select from the dropdown" prompt="Please select from the dropdown" sqref="G2:G1048576" xr:uid="{0A9DBD8E-98B5-417D-8BBE-275D4F7BAF2E}">
-      <formula1>#REF!</formula1>
-    </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="H2" r:id="rId1" xr:uid="{7B834616-30C9-4ABF-A492-9F49BDC23D50}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:IV59"/>
+  <dimension ref="A1:IV54"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="42.109375" style="2" customWidth="1"/>
@@ -5963,16 +6000,16 @@
     </row>
     <row r="2" spans="1:256">
       <c r="A2" s="24" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="B2" s="14"/>
     </row>
     <row r="3" spans="1:256" ht="14.4">
       <c r="A3" s="15" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="C3" s="4"/>
       <c r="D3" s="4"/>
@@ -6232,7 +6269,7 @@
     <row r="4" spans="1:256" ht="14.4">
       <c r="A4" s="17"/>
       <c r="B4" s="16" t="s">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -6492,7 +6529,7 @@
     <row r="5" spans="1:256" ht="14.4">
       <c r="A5" s="17"/>
       <c r="B5" s="16" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="C5"/>
       <c r="D5"/>
@@ -6751,34 +6788,34 @@
     </row>
     <row r="6" spans="1:256">
       <c r="A6" s="19" t="s">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="B6" s="18"/>
     </row>
     <row r="7" spans="1:256">
       <c r="A7" s="15" t="s">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="B7" s="18"/>
     </row>
     <row r="8" spans="1:256">
       <c r="A8" s="15" t="s">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="B8" s="18"/>
     </row>
     <row r="9" spans="1:256">
       <c r="A9" s="17" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="B9" s="18"/>
     </row>
     <row r="10" spans="1:256" ht="16.5" customHeight="1">
       <c r="A10" s="21" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="C10"/>
       <c r="D10"/>
@@ -7038,7 +7075,7 @@
     <row r="11" spans="1:256" ht="15" customHeight="1">
       <c r="A11" s="21"/>
       <c r="B11" s="22" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="C11"/>
       <c r="D11"/>
@@ -7298,7 +7335,7 @@
     <row r="12" spans="1:256" ht="15" customHeight="1">
       <c r="A12" s="32"/>
       <c r="B12" s="23" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="C12"/>
       <c r="D12"/>
@@ -7557,7 +7594,7 @@
     </row>
     <row r="13" spans="1:256" ht="15" customHeight="1">
       <c r="A13" s="28" t="s">
-        <v>124</v>
+        <v>111</v>
       </c>
       <c r="B13" s="29"/>
       <c r="C13"/>
@@ -8353,10 +8390,10 @@
         <v>5</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="D17" s="7" t="s">
         <v>6</v>
@@ -8368,7 +8405,7 @@
         <v>7</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="C18" s="7" t="s">
         <v>8</v>
@@ -8383,7 +8420,7 @@
         <v>9</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="C19" s="7" t="s">
         <v>10</v>
@@ -8398,7 +8435,7 @@
         <v>11</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>81</v>
+        <v>70</v>
       </c>
       <c r="C20" s="7" t="s">
         <v>10</v>
@@ -8413,7 +8450,7 @@
         <v>12</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="C21" s="7" t="s">
         <v>10</v>
@@ -8428,7 +8465,7 @@
         <v>13</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>76</v>
+        <v>65</v>
       </c>
       <c r="C22" s="7" t="s">
         <v>10</v>
@@ -8440,10 +8477,10 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="8" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="C23" s="7"/>
       <c r="D23" s="7" t="s">
@@ -8455,10 +8492,10 @@
     </row>
     <row r="24" spans="1:5" ht="69">
       <c r="A24" s="8" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="C24" s="7" t="s">
         <v>8</v>
@@ -8470,13 +8507,13 @@
     </row>
     <row r="25" spans="1:5" ht="72.900000000000006" customHeight="1">
       <c r="A25" s="12" t="s">
-        <v>129</v>
+        <v>116</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>130</v>
+        <v>117</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>128</v>
+        <v>115</v>
       </c>
       <c r="D25" s="10" t="s">
         <v>21</v>
@@ -8488,7 +8525,7 @@
         <v>30</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="C26" s="10" t="s">
         <v>31</v>
@@ -8500,10 +8537,10 @@
     </row>
     <row r="27" spans="1:5" s="3" customFormat="1" ht="27.6">
       <c r="A27" s="10" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="C27" s="10" t="s">
         <v>31</v>
@@ -8518,7 +8555,7 @@
         <v>32</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="C28" s="10"/>
       <c r="D28" s="10" t="s">
@@ -8530,10 +8567,10 @@
     </row>
     <row r="29" spans="1:5" ht="110.4">
       <c r="A29" s="10" t="s">
-        <v>126</v>
+        <v>113</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>131</v>
+        <v>118</v>
       </c>
       <c r="C29" s="7" t="s">
         <v>8</v>
@@ -8545,10 +8582,10 @@
     </row>
     <row r="30" spans="1:5" ht="124.2">
       <c r="A30" s="11" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>132</v>
+        <v>119</v>
       </c>
       <c r="C30" s="7" t="s">
         <v>15</v>
@@ -8563,13 +8600,13 @@
         <v>14</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="C31" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="E31" s="7"/>
     </row>
@@ -8578,13 +8615,13 @@
         <v>16</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="C32" s="7" t="s">
         <v>17</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="E32" s="7"/>
     </row>
@@ -8593,13 +8630,13 @@
         <v>18</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="C33" s="7" t="s">
         <v>19</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="E33" s="7"/>
     </row>
@@ -8608,13 +8645,13 @@
         <v>20</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="C34" s="7" t="s">
         <v>8</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="E34" s="7"/>
     </row>
@@ -8623,11 +8660,11 @@
         <v>22</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="C35" s="7"/>
       <c r="D35" s="9" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="E35" s="7"/>
     </row>
@@ -8636,7 +8673,7 @@
         <v>24</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="C36" s="7" t="s">
         <v>15</v>
@@ -8648,13 +8685,13 @@
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="7" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="D37" s="7" t="s">
         <v>21</v>
@@ -8663,74 +8700,74 @@
     </row>
     <row r="38" spans="1:5" ht="55.2">
       <c r="A38" s="10" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="B38" s="11" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="C38" s="10" t="s">
         <v>10</v>
       </c>
       <c r="D38" s="7" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="E38" s="8"/>
     </row>
     <row r="39" spans="1:5" ht="60.75" customHeight="1">
       <c r="A39" s="10" t="s">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="B39" s="11" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="C39" s="10" t="s">
         <v>10</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="E39" s="8"/>
     </row>
     <row r="40" spans="1:5" ht="16.5" customHeight="1">
       <c r="A40" s="10" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="B40" s="11" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="D40" s="7" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="E40" s="8"/>
     </row>
     <row r="41" spans="1:5" ht="18.75" customHeight="1">
       <c r="A41" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="B41" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="C41" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="D41" s="7" t="s">
         <v>60</v>
-      </c>
-      <c r="B41" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="C41" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="D41" s="7" t="s">
-        <v>71</v>
       </c>
       <c r="E41" s="8"/>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" s="10" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>108</v>
+        <v>97</v>
       </c>
       <c r="C42" s="7"/>
       <c r="D42" s="7" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="E42" s="7" t="s">
         <v>33</v>
@@ -8741,13 +8778,13 @@
         <v>25</v>
       </c>
       <c r="B43" s="11" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="C43" s="10" t="s">
         <v>15</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
       <c r="E43" s="8"/>
     </row>
@@ -8756,13 +8793,13 @@
         <v>26</v>
       </c>
       <c r="B44" s="11" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="C44" s="10" t="s">
         <v>17</v>
       </c>
       <c r="D44" s="11" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="E44" s="8"/>
     </row>
@@ -8771,13 +8808,13 @@
         <v>27</v>
       </c>
       <c r="B45" s="11" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="C45" s="10" t="s">
         <v>19</v>
       </c>
       <c r="D45" s="11" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="E45" s="8"/>
     </row>
@@ -8786,13 +8823,13 @@
         <v>28</v>
       </c>
       <c r="B46" s="11" t="s">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="C46" s="10" t="s">
         <v>8</v>
       </c>
       <c r="D46" s="11" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="E46" s="8"/>
     </row>
@@ -8801,13 +8838,13 @@
         <v>29</v>
       </c>
       <c r="B47" s="11" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="C47" s="10" t="s">
         <v>23</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="E47" s="8"/>
     </row>
@@ -8816,7 +8853,7 @@
         <v>34</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="C48" s="7"/>
       <c r="D48" s="7" t="s">
@@ -8892,13 +8929,13 @@
     </row>
     <row r="53" spans="1:5" ht="27.6">
       <c r="A53" s="7" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="B53" s="9" t="s">
-        <v>125</v>
+        <v>112</v>
       </c>
       <c r="C53" s="27" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="D53" s="7" t="s">
         <v>6</v>
@@ -8907,91 +8944,16 @@
     </row>
     <row r="54" spans="1:5" ht="47.1" customHeight="1">
       <c r="A54" s="9" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="B54" s="9" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="C54" s="7"/>
       <c r="D54" s="7" t="s">
         <v>40</v>
       </c>
       <c r="E54" s="7"/>
-    </row>
-    <row r="55" spans="1:5" ht="32.4" customHeight="1">
-      <c r="A55" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="B55" s="9" t="s">
-        <v>123</v>
-      </c>
-      <c r="C55" s="7"/>
-      <c r="D55" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="E55" s="7"/>
-    </row>
-    <row r="56" spans="1:5" ht="29.4" customHeight="1">
-      <c r="A56" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="B56" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="C56" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="D56" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="E56" s="7"/>
-    </row>
-    <row r="57" spans="1:5" ht="27.6">
-      <c r="A57" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="B57" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="C57" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="D57" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="E57" s="7" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" ht="27.6">
-      <c r="A58" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="B58" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="C58" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="D58" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="E58" s="7"/>
-    </row>
-    <row r="59" spans="1:5" ht="27.6">
-      <c r="A59" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="B59" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="C59" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="D59" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="E59" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9009,17 +8971,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3fa6fcba-af30-41d8-8f68-e31b5968a495">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="053c2422-fdcd-43dd-8361-3405662cd81a" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101007A9270DE7CEABF4D85DD0FDC5F4B5B3A" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c4d3f5216d7c68a25ceaa840d8f85b77">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3fa6fcba-af30-41d8-8f68-e31b5968a495" xmlns:ns3="053c2422-fdcd-43dd-8361-3405662cd81a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="bc464f71de289bf05fb818f223d9a5e3" ns2:_="" ns3:_="">
     <xsd:import namespace="3fa6fcba-af30-41d8-8f68-e31b5968a495"/>
@@ -9274,6 +9225,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3fa6fcba-af30-41d8-8f68-e31b5968a495">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="053c2422-fdcd-43dd-8361-3405662cd81a" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD3CCCF7-A5F0-457C-9882-571AC06F33B6}">
   <ds:schemaRefs>
@@ -9283,23 +9245,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{712C62DF-5115-4C46-B7B4-505402D5535E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="3fa6fcba-af30-41d8-8f68-e31b5968a495"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="053c2422-fdcd-43dd-8361-3405662cd81a"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B7C30678-80F6-4412-9C01-7CBD0F38B822}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9316,4 +9261,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{712C62DF-5115-4C46-B7B4-505402D5535E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="3fa6fcba-af30-41d8-8f68-e31b5968a495"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="053c2422-fdcd-43dd-8361-3405662cd81a"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>